<commit_message>
Added extn and corresponding change to Attachment
</commit_message>
<xml_diff>
--- a/314e-ig/output/StructureDefinition-attachment-314e.xlsx
+++ b/314e-ig/output/StructureDefinition-attachment-314e.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="182">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-13T11:15:06+05:30</t>
+    <t>2026-05-13T15:29:14+05:30</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -380,6 +380,24 @@
 This extension allows multiple tags to be associated with an
 Attachment for workflow, classification, indexing, or retrieval
 purposes.</t>
+  </si>
+  <si>
+    <t>Attachment.extension:helperFile</t>
+  </si>
+  <si>
+    <t>helperFile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extension {http://314e.com/fhir/StructureDefinition/attachment-helperFile}
+</t>
+  </si>
+  <si>
+    <t>Helper file associated with the attachment</t>
+  </si>
+  <si>
+    <t>Provides the path or filename of an auxiliary/helper file required
+for interpretation, transformation, rendering, or processing of
+the attachment content.</t>
   </si>
   <si>
     <t>Attachment.contentType</t>
@@ -880,7 +898,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AL14"/>
+  <dimension ref="A1:AL15"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="36.953125" customWidth="true" bestFit="true"/>
@@ -1581,9 +1599,11 @@
         <v>114</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>114</v>
-      </c>
-      <c r="C7" s="2"/>
+        <v>93</v>
+      </c>
+      <c r="C7" t="s" s="2">
+        <v>115</v>
+      </c>
       <c r="D7" t="s" s="2">
         <v>20</v>
       </c>
@@ -1601,7 +1621,7 @@
         <v>20</v>
       </c>
       <c r="J7" t="s" s="2">
-        <v>115</v>
+        <v>20</v>
       </c>
       <c r="K7" t="s" s="2">
         <v>116</v>
@@ -1613,9 +1633,7 @@
         <v>118</v>
       </c>
       <c r="N7" s="2"/>
-      <c r="O7" t="s" s="2">
-        <v>119</v>
-      </c>
+      <c r="O7" s="2"/>
       <c r="P7" t="s" s="2">
         <v>20</v>
       </c>
@@ -1627,7 +1645,7 @@
         <v>20</v>
       </c>
       <c r="T7" t="s" s="2">
-        <v>120</v>
+        <v>20</v>
       </c>
       <c r="U7" t="s" s="2">
         <v>20</v>
@@ -1639,13 +1657,13 @@
         <v>20</v>
       </c>
       <c r="X7" t="s" s="2">
-        <v>121</v>
+        <v>20</v>
       </c>
       <c r="Y7" t="s" s="2">
-        <v>122</v>
+        <v>20</v>
       </c>
       <c r="Z7" t="s" s="2">
-        <v>123</v>
+        <v>20</v>
       </c>
       <c r="AA7" t="s" s="2">
         <v>20</v>
@@ -1663,33 +1681,33 @@
         <v>20</v>
       </c>
       <c r="AF7" t="s" s="2">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="AG7" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH7" t="s" s="2">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="AI7" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AJ7" t="s" s="2">
-        <v>124</v>
+        <v>103</v>
       </c>
       <c r="AK7" t="s" s="2">
-        <v>125</v>
+        <v>20</v>
       </c>
       <c r="AL7" t="s" s="2">
-        <v>126</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" t="s" s="2">
@@ -1709,20 +1727,20 @@
         <v>20</v>
       </c>
       <c r="J8" t="s" s="2">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="K8" t="s" s="2">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="L8" t="s" s="2">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="M8" t="s" s="2">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="N8" s="2"/>
       <c r="O8" t="s" s="2">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="P8" t="s" s="2">
         <v>20</v>
@@ -1735,7 +1753,7 @@
         <v>20</v>
       </c>
       <c r="T8" t="s" s="2">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="U8" t="s" s="2">
         <v>20</v>
@@ -1747,13 +1765,13 @@
         <v>20</v>
       </c>
       <c r="X8" t="s" s="2">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="Y8" t="s" s="2">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="Z8" t="s" s="2">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="AA8" t="s" s="2">
         <v>20</v>
@@ -1771,7 +1789,7 @@
         <v>20</v>
       </c>
       <c r="AF8" t="s" s="2">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="AG8" t="s" s="2">
         <v>76</v>
@@ -1783,21 +1801,21 @@
         <v>20</v>
       </c>
       <c r="AJ8" t="s" s="2">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="AK8" t="s" s="2">
-        <v>20</v>
+        <v>130</v>
       </c>
       <c r="AL8" t="s" s="2">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" t="s" s="2">
@@ -1808,7 +1826,7 @@
         <v>76</v>
       </c>
       <c r="G9" t="s" s="2">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="H9" t="s" s="2">
         <v>20</v>
@@ -1817,22 +1835,20 @@
         <v>20</v>
       </c>
       <c r="J9" t="s" s="2">
-        <v>20</v>
+        <v>120</v>
       </c>
       <c r="K9" t="s" s="2">
-        <v>137</v>
+        <v>121</v>
       </c>
       <c r="L9" t="s" s="2">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="M9" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="N9" t="s" s="2">
-        <v>140</v>
-      </c>
+        <v>134</v>
+      </c>
+      <c r="N9" s="2"/>
       <c r="O9" t="s" s="2">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="P9" t="s" s="2">
         <v>20</v>
@@ -1845,7 +1861,7 @@
         <v>20</v>
       </c>
       <c r="T9" t="s" s="2">
-        <v>20</v>
+        <v>136</v>
       </c>
       <c r="U9" t="s" s="2">
         <v>20</v>
@@ -1857,13 +1873,13 @@
         <v>20</v>
       </c>
       <c r="X9" t="s" s="2">
-        <v>20</v>
+        <v>137</v>
       </c>
       <c r="Y9" t="s" s="2">
-        <v>20</v>
+        <v>138</v>
       </c>
       <c r="Z9" t="s" s="2">
-        <v>20</v>
+        <v>139</v>
       </c>
       <c r="AA9" t="s" s="2">
         <v>20</v>
@@ -1881,7 +1897,7 @@
         <v>20</v>
       </c>
       <c r="AF9" t="s" s="2">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="AG9" t="s" s="2">
         <v>76</v>
@@ -1893,21 +1909,21 @@
         <v>20</v>
       </c>
       <c r="AJ9" t="s" s="2">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="AK9" t="s" s="2">
-        <v>142</v>
+        <v>20</v>
       </c>
       <c r="AL9" t="s" s="2">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" t="s" s="2">
@@ -1915,10 +1931,10 @@
       </c>
       <c r="E10" s="2"/>
       <c r="F10" t="s" s="2">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="G10" t="s" s="2">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="H10" t="s" s="2">
         <v>20</v>
@@ -1927,22 +1943,22 @@
         <v>20</v>
       </c>
       <c r="J10" t="s" s="2">
-        <v>115</v>
+        <v>20</v>
       </c>
       <c r="K10" t="s" s="2">
+        <v>142</v>
+      </c>
+      <c r="L10" t="s" s="2">
+        <v>143</v>
+      </c>
+      <c r="M10" t="s" s="2">
+        <v>144</v>
+      </c>
+      <c r="N10" t="s" s="2">
         <v>145</v>
       </c>
-      <c r="L10" t="s" s="2">
+      <c r="O10" t="s" s="2">
         <v>146</v>
-      </c>
-      <c r="M10" t="s" s="2">
-        <v>147</v>
-      </c>
-      <c r="N10" t="s" s="2">
-        <v>148</v>
-      </c>
-      <c r="O10" t="s" s="2">
-        <v>149</v>
       </c>
       <c r="P10" t="s" s="2">
         <v>20</v>
@@ -1955,7 +1971,7 @@
         <v>20</v>
       </c>
       <c r="T10" t="s" s="2">
-        <v>150</v>
+        <v>20</v>
       </c>
       <c r="U10" t="s" s="2">
         <v>20</v>
@@ -1991,7 +2007,7 @@
         <v>20</v>
       </c>
       <c r="AF10" t="s" s="2">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="AG10" t="s" s="2">
         <v>76</v>
@@ -2003,21 +2019,21 @@
         <v>20</v>
       </c>
       <c r="AJ10" t="s" s="2">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="AK10" t="s" s="2">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="AL10" t="s" s="2">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
@@ -2025,7 +2041,7 @@
       </c>
       <c r="E11" s="2"/>
       <c r="F11" t="s" s="2">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="G11" t="s" s="2">
         <v>87</v>
@@ -2037,22 +2053,22 @@
         <v>20</v>
       </c>
       <c r="J11" t="s" s="2">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="K11" t="s" s="2">
+        <v>150</v>
+      </c>
+      <c r="L11" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="M11" t="s" s="2">
+        <v>152</v>
+      </c>
+      <c r="N11" t="s" s="2">
+        <v>153</v>
+      </c>
+      <c r="O11" t="s" s="2">
         <v>154</v>
-      </c>
-      <c r="L11" t="s" s="2">
-        <v>155</v>
-      </c>
-      <c r="M11" t="s" s="2">
-        <v>156</v>
-      </c>
-      <c r="N11" t="s" s="2">
-        <v>157</v>
-      </c>
-      <c r="O11" t="s" s="2">
-        <v>158</v>
       </c>
       <c r="P11" t="s" s="2">
         <v>20</v>
@@ -2065,7 +2081,7 @@
         <v>20</v>
       </c>
       <c r="T11" t="s" s="2">
-        <v>20</v>
+        <v>155</v>
       </c>
       <c r="U11" t="s" s="2">
         <v>20</v>
@@ -2101,7 +2117,7 @@
         <v>20</v>
       </c>
       <c r="AF11" t="s" s="2">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="AG11" t="s" s="2">
         <v>76</v>
@@ -2113,21 +2129,21 @@
         <v>20</v>
       </c>
       <c r="AJ11" t="s" s="2">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="AK11" t="s" s="2">
-        <v>20</v>
+        <v>156</v>
       </c>
       <c r="AL11" t="s" s="2">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
@@ -2147,22 +2163,22 @@
         <v>20</v>
       </c>
       <c r="J12" t="s" s="2">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="K12" t="s" s="2">
-        <v>137</v>
+        <v>159</v>
       </c>
       <c r="L12" t="s" s="2">
+        <v>160</v>
+      </c>
+      <c r="M12" t="s" s="2">
         <v>161</v>
       </c>
-      <c r="M12" t="s" s="2">
+      <c r="N12" t="s" s="2">
         <v>162</v>
       </c>
-      <c r="N12" t="s" s="2">
+      <c r="O12" t="s" s="2">
         <v>163</v>
-      </c>
-      <c r="O12" t="s" s="2">
-        <v>164</v>
       </c>
       <c r="P12" t="s" s="2">
         <v>20</v>
@@ -2211,7 +2227,7 @@
         <v>20</v>
       </c>
       <c r="AF12" t="s" s="2">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>76</v>
@@ -2223,21 +2239,21 @@
         <v>20</v>
       </c>
       <c r="AJ12" t="s" s="2">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="AK12" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL12" t="s" s="2">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2257,18 +2273,20 @@
         <v>20</v>
       </c>
       <c r="J13" t="s" s="2">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>88</v>
+        <v>142</v>
       </c>
       <c r="L13" t="s" s="2">
+        <v>166</v>
+      </c>
+      <c r="M13" t="s" s="2">
         <v>167</v>
       </c>
-      <c r="M13" t="s" s="2">
+      <c r="N13" t="s" s="2">
         <v>168</v>
       </c>
-      <c r="N13" s="2"/>
       <c r="O13" t="s" s="2">
         <v>169</v>
       </c>
@@ -2283,7 +2301,7 @@
         <v>20</v>
       </c>
       <c r="T13" t="s" s="2">
-        <v>170</v>
+        <v>20</v>
       </c>
       <c r="U13" t="s" s="2">
         <v>20</v>
@@ -2319,7 +2337,7 @@
         <v>20</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>76</v>
@@ -2331,21 +2349,21 @@
         <v>20</v>
       </c>
       <c r="AJ13" t="s" s="2">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="AK13" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL13" t="s" s="2">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -2365,20 +2383,20 @@
         <v>20</v>
       </c>
       <c r="J14" t="s" s="2">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="K14" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="L14" t="s" s="2">
+        <v>172</v>
+      </c>
+      <c r="M14" t="s" s="2">
         <v>173</v>
-      </c>
-      <c r="L14" t="s" s="2">
-        <v>174</v>
-      </c>
-      <c r="M14" t="s" s="2">
-        <v>175</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" t="s" s="2">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="P14" t="s" s="2">
         <v>20</v>
@@ -2391,7 +2409,7 @@
         <v>20</v>
       </c>
       <c r="T14" t="s" s="2">
-        <v>20</v>
+        <v>175</v>
       </c>
       <c r="U14" t="s" s="2">
         <v>20</v>
@@ -2427,7 +2445,7 @@
         <v>20</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>76</v>
@@ -2439,13 +2457,121 @@
         <v>20</v>
       </c>
       <c r="AJ14" t="s" s="2">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="AK14" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL14" t="s" s="2">
-        <v>159</v>
+        <v>176</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="B15" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="C15" s="2"/>
+      <c r="D15" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="E15" s="2"/>
+      <c r="F15" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G15" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H15" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="I15" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="J15" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="K15" t="s" s="2">
+        <v>178</v>
+      </c>
+      <c r="L15" t="s" s="2">
+        <v>179</v>
+      </c>
+      <c r="M15" t="s" s="2">
+        <v>180</v>
+      </c>
+      <c r="N15" s="2"/>
+      <c r="O15" t="s" s="2">
+        <v>181</v>
+      </c>
+      <c r="P15" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Q15" s="2"/>
+      <c r="R15" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="S15" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="T15" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="U15" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="V15" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="W15" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="X15" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Y15" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Z15" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AA15" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AB15" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AC15" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AD15" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AE15" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AF15" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="AG15" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH15" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI15" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AJ15" t="s" s="2">
+        <v>129</v>
+      </c>
+      <c r="AK15" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AL15" t="s" s="2">
+        <v>164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updates to the attachment datatype, getting rid of inlinedatasavedasfile extn., adding codesystem and valueset for attachment tag extension and updates to the extension descriptions in the quantity datatype
</commit_message>
<xml_diff>
--- a/314e-ig/output/StructureDefinition-attachment-314e.xlsx
+++ b/314e-ig/output/StructureDefinition-attachment-314e.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="177">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-13T15:29:14+05:30</t>
+    <t>2026-05-15T09:21:03+05:30</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -85,9 +85,11 @@
 SHALL never be populated.
 All attachment content SHALL be externalized into object storage
 and referenced using Attachment.url.
-If content originated as inline data/blob content and was later
-saved externally, the extension
-attachment-inlineDataSavedAsFile SHALL be used to indicate this.</t>
+If attachment content originated as inline data/blob content
+and was subsequently externalized into object storage, the
+Attachment SHALL carry the tag
+'inline-data-externalized-to-file' using the attachment-tag
+extension.</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -342,27 +344,6 @@
 ext-1:Must have either extensions or value[x], not both {extension.exists() != value.exists()}</t>
   </si>
   <si>
-    <t>Attachment.extension:inlineDataSavedAsFile</t>
-  </si>
-  <si>
-    <t>inlineDataSavedAsFile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extension {http://314e.com/fhir/StructureDefinition/attachment-inlineDataSavedAsFile}
-</t>
-  </si>
-  <si>
-    <t>Indicates originally-inline content externalized into object storage</t>
-  </si>
-  <si>
-    <t>Indicates that the Attachment content was originally available
-as inline data/blob content but has been externalized and saved
-as a file in object storage, with the Attachment.url carrying
-the storage location.
-If this extension is absent, the content SHALL be assumed to
-have originated as an external file rather than inline data.</t>
-  </si>
-  <si>
     <t>Attachment.extension:tag</t>
   </si>
   <si>
@@ -376,10 +357,10 @@
     <t>Semantic categorization tag associated with the attachment</t>
   </si>
   <si>
-    <t>A categorization or tagging label associated with an Attachment.
+    <t>A categorization or semantic tag associated with an Attachment.
 This extension allows multiple tags to be associated with an
-Attachment for workflow, classification, indexing, or retrieval
-purposes.</t>
+Attachment for workflow, classification, indexing, retrieval,
+processing, or application behavior purposes.</t>
   </si>
   <si>
     <t>Attachment.extension:helperFile</t>
@@ -505,7 +486,9 @@
     <t>Object storage path or external attachment location</t>
   </si>
   <si>
-    <t>Reference/path to the externally stored attachment content.</t>
+    <t>Reference/path to the externally stored attachment content. Inline binary data in 
+Attachment.data SHALL NOT be populated. Inline content SHALL instead be persisted 
+externally, referenced using this url element, and tagged as 'inline-data-externalized-to-file'.</t>
   </si>
   <si>
     <t>If both data and url are provided, the url SHALL point to the same content as the data contains. Urls may be relative references or may reference transient locations such as a wrapping envelope using cid: though this has ramifications for using signatures. Relative URLs are interpreted relative to the service url, like a resource reference, rather than relative to the resource itself. If a URL is provided, it SHALL resolve to actual data.</t>
@@ -898,12 +881,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AL15"/>
+  <dimension ref="A1:AL14"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="36.953125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="27.27734375" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="21.0859375" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="18.578125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="3" max="3" width="9.984375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="11.10546875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.29296875" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.21484375" customWidth="true" bestFit="true"/>
@@ -911,7 +894,7 @@
     <col min="8" max="8" width="13.1171875" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="10.75390625" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="71.87109375" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="62.1953125" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -1396,7 +1379,7 @@
         <v>76</v>
       </c>
       <c r="G5" t="s" s="2">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="H5" t="s" s="2">
         <v>20</v>
@@ -1504,7 +1487,7 @@
         <v>76</v>
       </c>
       <c r="G6" t="s" s="2">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="H6" t="s" s="2">
         <v>20</v>
@@ -1599,11 +1582,9 @@
         <v>114</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="C7" t="s" s="2">
-        <v>115</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="C7" s="2"/>
       <c r="D7" t="s" s="2">
         <v>20</v>
       </c>
@@ -1621,7 +1602,7 @@
         <v>20</v>
       </c>
       <c r="J7" t="s" s="2">
-        <v>20</v>
+        <v>115</v>
       </c>
       <c r="K7" t="s" s="2">
         <v>116</v>
@@ -1633,7 +1614,9 @@
         <v>118</v>
       </c>
       <c r="N7" s="2"/>
-      <c r="O7" s="2"/>
+      <c r="O7" t="s" s="2">
+        <v>119</v>
+      </c>
       <c r="P7" t="s" s="2">
         <v>20</v>
       </c>
@@ -1645,7 +1628,7 @@
         <v>20</v>
       </c>
       <c r="T7" t="s" s="2">
-        <v>20</v>
+        <v>120</v>
       </c>
       <c r="U7" t="s" s="2">
         <v>20</v>
@@ -1657,13 +1640,13 @@
         <v>20</v>
       </c>
       <c r="X7" t="s" s="2">
-        <v>20</v>
+        <v>121</v>
       </c>
       <c r="Y7" t="s" s="2">
-        <v>20</v>
+        <v>122</v>
       </c>
       <c r="Z7" t="s" s="2">
-        <v>20</v>
+        <v>123</v>
       </c>
       <c r="AA7" t="s" s="2">
         <v>20</v>
@@ -1681,33 +1664,33 @@
         <v>20</v>
       </c>
       <c r="AF7" t="s" s="2">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="AG7" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH7" t="s" s="2">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="AI7" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AJ7" t="s" s="2">
-        <v>103</v>
+        <v>124</v>
       </c>
       <c r="AK7" t="s" s="2">
-        <v>20</v>
+        <v>125</v>
       </c>
       <c r="AL7" t="s" s="2">
-        <v>20</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" t="s" s="2">
@@ -1727,20 +1710,20 @@
         <v>20</v>
       </c>
       <c r="J8" t="s" s="2">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="K8" t="s" s="2">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="L8" t="s" s="2">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="M8" t="s" s="2">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="N8" s="2"/>
       <c r="O8" t="s" s="2">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="P8" t="s" s="2">
         <v>20</v>
@@ -1753,7 +1736,7 @@
         <v>20</v>
       </c>
       <c r="T8" t="s" s="2">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="U8" t="s" s="2">
         <v>20</v>
@@ -1765,31 +1748,31 @@
         <v>20</v>
       </c>
       <c r="X8" t="s" s="2">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="Y8" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="Z8" t="s" s="2">
+        <v>134</v>
+      </c>
+      <c r="AA8" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AB8" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AC8" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AD8" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AE8" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AF8" t="s" s="2">
         <v>127</v>
-      </c>
-      <c r="Z8" t="s" s="2">
-        <v>128</v>
-      </c>
-      <c r="AA8" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AB8" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AC8" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AD8" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AE8" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AF8" t="s" s="2">
-        <v>119</v>
       </c>
       <c r="AG8" t="s" s="2">
         <v>76</v>
@@ -1801,21 +1784,21 @@
         <v>20</v>
       </c>
       <c r="AJ8" t="s" s="2">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AK8" t="s" s="2">
-        <v>130</v>
+        <v>20</v>
       </c>
       <c r="AL8" t="s" s="2">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" t="s" s="2">
@@ -1826,7 +1809,7 @@
         <v>76</v>
       </c>
       <c r="G9" t="s" s="2">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="H9" t="s" s="2">
         <v>20</v>
@@ -1835,20 +1818,22 @@
         <v>20</v>
       </c>
       <c r="J9" t="s" s="2">
-        <v>120</v>
+        <v>20</v>
       </c>
       <c r="K9" t="s" s="2">
-        <v>121</v>
+        <v>137</v>
       </c>
       <c r="L9" t="s" s="2">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="M9" t="s" s="2">
-        <v>134</v>
-      </c>
-      <c r="N9" s="2"/>
+        <v>139</v>
+      </c>
+      <c r="N9" t="s" s="2">
+        <v>140</v>
+      </c>
       <c r="O9" t="s" s="2">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="P9" t="s" s="2">
         <v>20</v>
@@ -1861,43 +1846,43 @@
         <v>20</v>
       </c>
       <c r="T9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="U9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="V9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="W9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="X9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Y9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Z9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AA9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AB9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AC9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AD9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AE9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AF9" t="s" s="2">
         <v>136</v>
-      </c>
-      <c r="U9" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="V9" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="W9" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="X9" t="s" s="2">
-        <v>137</v>
-      </c>
-      <c r="Y9" t="s" s="2">
-        <v>138</v>
-      </c>
-      <c r="Z9" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="AA9" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AB9" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AC9" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AD9" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AE9" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AF9" t="s" s="2">
-        <v>132</v>
       </c>
       <c r="AG9" t="s" s="2">
         <v>76</v>
@@ -1909,21 +1894,21 @@
         <v>20</v>
       </c>
       <c r="AJ9" t="s" s="2">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AK9" t="s" s="2">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="AL9" t="s" s="2">
-        <v>140</v>
+        <v>143</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" t="s" s="2">
@@ -1931,10 +1916,10 @@
       </c>
       <c r="E10" s="2"/>
       <c r="F10" t="s" s="2">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="G10" t="s" s="2">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="H10" t="s" s="2">
         <v>20</v>
@@ -1943,22 +1928,22 @@
         <v>20</v>
       </c>
       <c r="J10" t="s" s="2">
-        <v>20</v>
+        <v>115</v>
       </c>
       <c r="K10" t="s" s="2">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="L10" t="s" s="2">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="M10" t="s" s="2">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="N10" t="s" s="2">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="O10" t="s" s="2">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="P10" t="s" s="2">
         <v>20</v>
@@ -1971,7 +1956,7 @@
         <v>20</v>
       </c>
       <c r="T10" t="s" s="2">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="U10" t="s" s="2">
         <v>20</v>
@@ -2007,7 +1992,7 @@
         <v>20</v>
       </c>
       <c r="AF10" t="s" s="2">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="AG10" t="s" s="2">
         <v>76</v>
@@ -2019,21 +2004,21 @@
         <v>20</v>
       </c>
       <c r="AJ10" t="s" s="2">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AK10" t="s" s="2">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="AL10" t="s" s="2">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
@@ -2041,7 +2026,7 @@
       </c>
       <c r="E11" s="2"/>
       <c r="F11" t="s" s="2">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="G11" t="s" s="2">
         <v>87</v>
@@ -2053,22 +2038,22 @@
         <v>20</v>
       </c>
       <c r="J11" t="s" s="2">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="K11" t="s" s="2">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="L11" t="s" s="2">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="M11" t="s" s="2">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="N11" t="s" s="2">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="O11" t="s" s="2">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="P11" t="s" s="2">
         <v>20</v>
@@ -2081,7 +2066,7 @@
         <v>20</v>
       </c>
       <c r="T11" t="s" s="2">
-        <v>155</v>
+        <v>20</v>
       </c>
       <c r="U11" t="s" s="2">
         <v>20</v>
@@ -2117,7 +2102,7 @@
         <v>20</v>
       </c>
       <c r="AF11" t="s" s="2">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="AG11" t="s" s="2">
         <v>76</v>
@@ -2129,21 +2114,21 @@
         <v>20</v>
       </c>
       <c r="AJ11" t="s" s="2">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AK11" t="s" s="2">
-        <v>156</v>
+        <v>20</v>
       </c>
       <c r="AL11" t="s" s="2">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
@@ -2163,22 +2148,22 @@
         <v>20</v>
       </c>
       <c r="J12" t="s" s="2">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="K12" t="s" s="2">
-        <v>159</v>
+        <v>137</v>
       </c>
       <c r="L12" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="N12" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="O12" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="P12" t="s" s="2">
         <v>20</v>
@@ -2227,7 +2212,7 @@
         <v>20</v>
       </c>
       <c r="AF12" t="s" s="2">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>76</v>
@@ -2239,21 +2224,21 @@
         <v>20</v>
       </c>
       <c r="AJ12" t="s" s="2">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AK12" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL12" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2273,20 +2258,18 @@
         <v>20</v>
       </c>
       <c r="J13" t="s" s="2">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>142</v>
+        <v>88</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>167</v>
-      </c>
-      <c r="N13" t="s" s="2">
         <v>168</v>
       </c>
+      <c r="N13" s="2"/>
       <c r="O13" t="s" s="2">
         <v>169</v>
       </c>
@@ -2301,7 +2284,7 @@
         <v>20</v>
       </c>
       <c r="T13" t="s" s="2">
-        <v>20</v>
+        <v>170</v>
       </c>
       <c r="U13" t="s" s="2">
         <v>20</v>
@@ -2337,7 +2320,7 @@
         <v>20</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>76</v>
@@ -2349,21 +2332,21 @@
         <v>20</v>
       </c>
       <c r="AJ13" t="s" s="2">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AK13" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL13" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -2383,20 +2366,20 @@
         <v>20</v>
       </c>
       <c r="J14" t="s" s="2">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>88</v>
+        <v>173</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" t="s" s="2">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="P14" t="s" s="2">
         <v>20</v>
@@ -2409,7 +2392,7 @@
         <v>20</v>
       </c>
       <c r="T14" t="s" s="2">
-        <v>175</v>
+        <v>20</v>
       </c>
       <c r="U14" t="s" s="2">
         <v>20</v>
@@ -2445,7 +2428,7 @@
         <v>20</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>76</v>
@@ -2457,121 +2440,13 @@
         <v>20</v>
       </c>
       <c r="AJ14" t="s" s="2">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AK14" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL14" t="s" s="2">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s" s="2">
-        <v>177</v>
-      </c>
-      <c r="B15" t="s" s="2">
-        <v>177</v>
-      </c>
-      <c r="C15" s="2"/>
-      <c r="D15" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="E15" s="2"/>
-      <c r="F15" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="G15" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H15" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="I15" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="J15" t="s" s="2">
-        <v>120</v>
-      </c>
-      <c r="K15" t="s" s="2">
-        <v>178</v>
-      </c>
-      <c r="L15" t="s" s="2">
-        <v>179</v>
-      </c>
-      <c r="M15" t="s" s="2">
-        <v>180</v>
-      </c>
-      <c r="N15" s="2"/>
-      <c r="O15" t="s" s="2">
-        <v>181</v>
-      </c>
-      <c r="P15" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="Q15" s="2"/>
-      <c r="R15" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="S15" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="T15" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="U15" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="V15" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="W15" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="X15" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="Y15" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="Z15" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AA15" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AB15" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AC15" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AD15" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AE15" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AF15" t="s" s="2">
-        <v>177</v>
-      </c>
-      <c r="AG15" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AH15" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI15" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AJ15" t="s" s="2">
-        <v>129</v>
-      </c>
-      <c r="AK15" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AL15" t="s" s="2">
-        <v>164</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>